<commit_message>
Added more aggregations for Kristin's DW variables
</commit_message>
<xml_diff>
--- a/config/CalSim3DataExtractionInitFile_v6.xlsx
+++ b/config/CalSim3DataExtractionInitFile_v6.xlsx
@@ -8,14 +8,25 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dino\COEQWAL\COEQWAL_GIT\COEQWAL_V3\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB5F606A-5ADC-4A28-A4F6-64CD552C8B2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DDFD737-C3E8-467E-9EE9-47D109593675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3120" yWindow="3075" windowWidth="17340" windowHeight="9990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Init" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -187,9 +198,6 @@
     <t>A2</t>
   </si>
   <si>
-    <t>O475</t>
-  </si>
-  <si>
     <t>Inflows Extraction Dir</t>
   </si>
   <si>
@@ -242,6 +250,9 @@
   </si>
   <si>
     <t>J101</t>
+  </si>
+  <si>
+    <t>O487</t>
   </si>
 </sst>
 </file>
@@ -579,14 +590,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="35.7109375" customWidth="1"/>
-    <col min="3" max="5" width="20.7109375" customWidth="1"/>
+    <col min="1" max="1" width="20.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="35.6640625" customWidth="1"/>
+    <col min="3" max="5" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -600,7 +611,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -608,15 +619,15 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
@@ -624,7 +635,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
@@ -635,10 +646,10 @@
         <v>11</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -649,10 +660,10 @@
         <v>14</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
@@ -663,10 +674,10 @@
         <v>17</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>18</v>
       </c>
@@ -677,10 +688,10 @@
         <v>20</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>21</v>
       </c>
@@ -691,10 +702,10 @@
         <v>23</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>24</v>
       </c>
@@ -705,10 +716,10 @@
         <v>26</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>27</v>
       </c>
@@ -719,10 +730,10 @@
         <v>29</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>30</v>
       </c>
@@ -730,7 +741,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>32</v>
       </c>
@@ -738,7 +749,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>34</v>
       </c>
@@ -746,7 +757,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>36</v>
       </c>
@@ -760,7 +771,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>40</v>
       </c>
@@ -768,7 +779,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>42</v>
       </c>
@@ -776,7 +787,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>44</v>
       </c>
@@ -784,7 +795,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>46</v>
       </c>
@@ -792,7 +803,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>48</v>
       </c>
@@ -800,7 +811,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>50</v>
       </c>
@@ -808,7 +819,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>52</v>
       </c>
@@ -819,45 +830,45 @@
         <v>54</v>
       </c>
       <c r="D22" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
+      <c r="B23" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B23" s="2" t="s">
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
+      <c r="B24" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B24" s="2" t="s">
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="1" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
+      <c r="B25" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B25" s="2" t="s">
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
+      <c r="B26" t="s">
         <v>62</v>
       </c>
-      <c r="B26" t="s">
+      <c r="C26" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="D26" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changed DW extraction not to delete intermediate columns, added one more variable
</commit_message>
<xml_diff>
--- a/config/CalSim3DataExtractionInitFile_v6.xlsx
+++ b/config/CalSim3DataExtractionInitFile_v6.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dino\COEQWAL\COEQWAL_GIT\COEQWAL_V3\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DDFD737-C3E8-467E-9EE9-47D109593675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90D0DF91-7383-4ECE-B179-8F899F865ACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3120" yWindow="3075" windowWidth="17340" windowHeight="9990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -252,7 +252,7 @@
     <t>J101</t>
   </si>
   <si>
-    <t>O487</t>
+    <t>O488</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
added 1 more aggregate DW variable
</commit_message>
<xml_diff>
--- a/config/CalSim3DataExtractionInitFile_v6.xlsx
+++ b/config/CalSim3DataExtractionInitFile_v6.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dino\COEQWAL\COEQWAL_GIT\COEQWAL_V3\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90D0DF91-7383-4ECE-B179-8F899F865ACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D971813-0781-47E6-A737-42B610786B72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3120" yWindow="3075" windowWidth="17340" windowHeight="9990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -252,7 +252,7 @@
     <t>J101</t>
   </si>
   <si>
-    <t>O488</t>
+    <t>O489</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
fixed latest DW variable issues
</commit_message>
<xml_diff>
--- a/config/CalSim3DataExtractionInitFile_v6.xlsx
+++ b/config/CalSim3DataExtractionInitFile_v6.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dino\COEQWAL\COEQWAL_GIT\COEQWAL_V3\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6EB505D-83B8-4285-BE75-8FDC3274F115}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8766CD5C-0C23-4F34-8806-07B6C8FC03EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -252,7 +252,7 @@
     <t>J101</t>
   </si>
   <si>
-    <t>O489</t>
+    <t>O486</t>
   </si>
 </sst>
 </file>

</xml_diff>